<commit_message>
Update Excel practice log
</commit_message>
<xml_diff>
--- a/data_practice.xlsx
+++ b/data_practice.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30621"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{07C49416-7D6D-4276-8661-4DE932D5DD6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BDCDEE18-584D-472C-9BBA-B4A39501D47D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" firstSheet="2" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="clean_wide" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
   </definedNames>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="693" r:id="rId6"/>
+    <pivotCache cacheId="421" r:id="rId6"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="55">
   <si>
     <t>Country Name</t>
   </si>
@@ -110,6 +110,69 @@
   </si>
   <si>
     <t>Why</t>
+  </si>
+  <si>
+    <t>Deleted the 3 title rows at the top and the 2 note rows at the bottom, so the header is in row 1</t>
+  </si>
+  <si>
+    <t>Pivots and filters need a clean header row</t>
+  </si>
+  <si>
+    <t>Deleted 2 blank rows and 2 duplicate rows (Mali and Nigeria, life expectancy). Data went from 28 to 24 rows</t>
+  </si>
+  <si>
+    <t>Duplicates would be counted twice in averages</t>
+  </si>
+  <si>
+    <t>Applied TRIM to remove extra spaces and replaced 'Ivory Coast' with "Côte d'Ivoire". Fixed "Côte D'Ivoire" (capital D) caused by PROPER</t>
+  </si>
+  <si>
+    <t>'Ghana ' and 'Ghana' would show up as two countries</t>
+  </si>
+  <si>
+    <t>One name per indicator, so filters and pivots work</t>
+  </si>
+  <si>
+    <t>Found and removed an invisible tab character at the start of 2 indicator cells (B14, B16) using the filter list</t>
+  </si>
+  <si>
+    <t>The tab made Excel see a fifth indicator</t>
+  </si>
+  <si>
+    <t>Removed the space from the '2019 ' header and made the year headers numbers</t>
+  </si>
+  <si>
+    <t>The header must match the other years</t>
+  </si>
+  <si>
+    <t>Replaced '..' (14 cells) and 'n/a' (5 cells) with empty cells</t>
+  </si>
+  <si>
+    <t>Text in a numeric column breaks averages</t>
+  </si>
+  <si>
+    <t>Converted numbers stored as text (with % signs and commas) into real numbers</t>
+  </si>
+  <si>
+    <t>Excel cannot add or average text</t>
+  </si>
+  <si>
+    <t>Reshaped from wide (years as columns) to long format with the TOCOL formula (Power Query is not available in Excel for the web), then pasted as values</t>
+  </si>
+  <si>
+    <t>A pivot table needs one value per row. Empty cells were skipped (144 cells became 116 values)</t>
+  </si>
+  <si>
+    <t>Built a pivot table of average GDP growth by country, filtered on the GDP indicator</t>
+  </si>
+  <si>
+    <t>To answer: which country grew fastest on average?</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>Cote d'Ivoire's average rests on only 2 data points, so it is less reliable than countries with 5 years</t>
   </si>
   <si>
     <t>Cleaning tasks (do them on a COPY of messy_data):</t>
@@ -167,12 +230,24 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -187,12 +262,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -245,6 +323,9 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
       <x14:pivotCacheDefinition/>
     </ext>
+    <ext xmlns:xlpdsc="http://schemas.microsoft.com/office/spreadsheetml/2026/pivotDataSourceClean" uri="{F4336242-56EE-4DD3-A5F7-E900642BF6E9}">
+      <xlpdsc:dataSourceClean>1</xlpdsc:dataSourceClean>
+    </ext>
   </extLst>
 </pivotCacheDefinition>
 </file>
@@ -951,7 +1032,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{295645FD-5449-486B-BFDC-5DA3286A3C4B}" name="PivotTable1" cacheId="693" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{295645FD-5449-486B-BFDC-5DA3286A3C4B}" name="PivotTable1" cacheId="421" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:B10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="4">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
@@ -3666,11 +3747,12 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F5DC5BA-1623-4F6A-BA57-00747A39C9D5}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="22.42578125" customWidth="1"/>
+    <col min="2" max="2" width="130.42578125" customWidth="1"/>
     <col min="3" max="3" width="23" customWidth="1"/>
+    <col min="4" max="4" width="84.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -3685,6 +3767,154 @@
       </c>
       <c r="D1" t="s">
         <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2">
+        <v>5</v>
+      </c>
+      <c r="D2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3">
+        <v>4</v>
+      </c>
+      <c r="D3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4">
+        <v>24</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5">
+        <v>24</v>
+      </c>
+      <c r="D5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8">
+        <v>19</v>
+      </c>
+      <c r="D8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9">
+        <v>12</v>
+      </c>
+      <c r="D9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10">
+        <v>116</v>
+      </c>
+      <c r="D10" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11">
+        <v>6</v>
+      </c>
+      <c r="D11" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -3702,57 +3932,57 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>23</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="2" t="s">
-        <v>24</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="2" t="s">
-        <v>25</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="2" t="s">
-        <v>26</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="2" t="s">
-        <v>27</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="2" t="s">
-        <v>28</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="2" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="2" t="s">
-        <v>30</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="2" t="s">
-        <v>31</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="2" t="s">
-        <v>32</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="2" t="s">
-        <v>33</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>